<commit_message>
Added do while loop to get the record for intended count
</commit_message>
<xml_diff>
--- a/bankingDetails.xlsx
+++ b/bankingDetails.xlsx
@@ -731,8 +731,8 @@
     <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
   <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1 1" defaultPivotStyle="PivotStylePreset2_Accent1 1">
-    <tableStyle name="TableStylePreset3_Accent1 1" pivot="0" count="0" xr9:uid="{FBFFAADA-AA3C-48CC-91E2-9B80F53C92D8}"/>
-    <tableStyle name="PivotStylePreset2_Accent1 1" table="0" count="0" xr9:uid="{36E815C3-BAB4-4116-B5FA-0E92F32B74B5}"/>
+    <tableStyle name="TableStylePreset3_Accent1 1" pivot="0" count="0" xr9:uid="{C846377E-2CB9-4EA5-98ED-E4FD23FF6235}"/>
+    <tableStyle name="PivotStylePreset2_Accent1 1" table="0" count="0" xr9:uid="{BA4BE3F5-3109-4957-810E-9D891527A3FC}"/>
   </tableStyles>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">

</xml_diff>